<commit_message>
COMMIT JUNE 17 FINAL
</commit_message>
<xml_diff>
--- a/FIFAScheduleResults.xlsx
+++ b/FIFAScheduleResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World Cup Betting/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="352" documentId="13_ncr:1_{AD0E7F59-3B0E-407E-93E9-FE21F83F93C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C913E90B-F68C-4667-A308-0B93A3E91F24}"/>
+  <xr:revisionPtr revIDLastSave="358" documentId="13_ncr:1_{AD0E7F59-3B0E-407E-93E9-FE21F83F93C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA4E0B95-30AC-46B0-A81D-2FE0CA6D3B35}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FIFA World Cup 2026" sheetId="1" r:id="rId1"/>
@@ -126,7 +126,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8168" uniqueCount="3813">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8170" uniqueCount="3814">
   <si>
     <t>Match</t>
   </si>
@@ -11565,6 +11565,9 @@
   </si>
   <si>
     <t>FRA10, FRA12, SEN20, FRA10</t>
+  </si>
+  <si>
+    <t>AUT18, JOR9, OG, AUT7</t>
   </si>
 </sst>
 </file>
@@ -14644,15 +14647,19 @@
       <c r="F57" s="135" t="s">
         <v>2379</v>
       </c>
-      <c r="G57" s="204"/>
-      <c r="H57" s="21"/>
-      <c r="I57" t="e" cm="1">
+      <c r="G57" s="204" t="s">
+        <v>3809</v>
+      </c>
+      <c r="H57" s="21" t="s">
+        <v>3813</v>
+      </c>
+      <c r="I57" t="str" cm="1">
         <f t="array" ref="I57">_xlfn.IFS(LEFT(G57,1)-RIGHT(G57,1) &gt; 0, "W1",LEFT(G57,1)-RIGHT(G57,1) = 0, "D",LEFT(G57,1)-RIGHT(G57,1) &lt; 0, "W2", ISBLANK(G57), "")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J57" s="144" t="e">
+        <v>W1</v>
+      </c>
+      <c r="J57" s="144">
         <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
7 on 8 bets
</commit_message>
<xml_diff>
--- a/FIFAScheduleResults.xlsx
+++ b/FIFAScheduleResults.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World Cup Betting/World-Cup-betting/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="388" documentId="13_ncr:1_{AD0E7F59-3B0E-407E-93E9-FE21F83F93C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85ACAC5D-7F57-4CA4-834F-E2518EEEFC10}"/>
+  <xr:revisionPtr revIDLastSave="389" documentId="13_ncr:1_{AD0E7F59-3B0E-407E-93E9-FE21F83F93C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D4D8271-5994-481D-8266-3890DD250E76}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FIFA World Cup 2026" sheetId="1" r:id="rId1"/>
@@ -12714,7 +12714,7 @@
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="15.81640625" customWidth="1"/>
     <col min="7" max="7" width="30" style="143" customWidth="1"/>
-    <col min="8" max="8" width="30" style="163" customWidth="1"/>
+    <col min="8" max="8" width="38.08984375" style="163" customWidth="1"/>
     <col min="9" max="9" width="20.7265625" customWidth="1"/>
     <col min="10" max="10" width="19.7265625" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Last 2nd round game
</commit_message>
<xml_diff>
--- a/FIFAScheduleResults.xlsx
+++ b/FIFAScheduleResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="450" documentId="13_ncr:1_{AD0E7F59-3B0E-407E-93E9-FE21F83F93C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{549EB84A-1893-47BD-BE4C-5B84FAE236D2}"/>
+  <xr:revisionPtr revIDLastSave="460" documentId="13_ncr:1_{AD0E7F59-3B0E-407E-93E9-FE21F83F93C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{577A8126-5436-4E83-AAE9-8E2303267153}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FIFA World Cup 2026" sheetId="1" r:id="rId1"/>
@@ -126,7 +126,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8216" uniqueCount="3843">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8223" uniqueCount="3847">
   <si>
     <t>Match</t>
   </si>
@@ -11655,6 +11655,18 @@
   </si>
   <si>
     <t>1-2</t>
+  </si>
+  <si>
+    <t>5-0</t>
+  </si>
+  <si>
+    <t>COL2</t>
+  </si>
+  <si>
+    <t>HRV11</t>
+  </si>
+  <si>
+    <t>POR7, POR25, POR7,OG, POR17</t>
   </si>
 </sst>
 </file>
@@ -14864,15 +14876,19 @@
       <c r="F64" s="136" t="s">
         <v>2386</v>
       </c>
-      <c r="G64" s="156"/>
-      <c r="H64" s="22"/>
-      <c r="I64" s="22" t="e" cm="1">
+      <c r="G64" s="156" t="s">
+        <v>3843</v>
+      </c>
+      <c r="H64" s="22" t="s">
+        <v>3846</v>
+      </c>
+      <c r="I64" s="22" t="str" cm="1">
         <f t="array" ref="I64">_xlfn.IFS(LEFT(G64,1)-RIGHT(G64,1) &gt; 0, "W1",LEFT(G64,1)-RIGHT(G64,1) = 0, "D",LEFT(G64,1)-RIGHT(G64,1) &lt; 0, "W2", ISBLANK(G64), "")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J64" s="23" t="e">
+        <v>W1</v>
+      </c>
+      <c r="J64" s="23">
         <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+        <v>5</v>
       </c>
     </row>
     <row r="65" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -14894,15 +14910,19 @@
       <c r="F65" s="136" t="s">
         <v>2387</v>
       </c>
-      <c r="G65" s="156"/>
-      <c r="H65" s="22"/>
-      <c r="I65" s="22" t="e" cm="1">
+      <c r="G65" s="156" t="s">
+        <v>2478</v>
+      </c>
+      <c r="H65" s="22" t="s">
+        <v>3844</v>
+      </c>
+      <c r="I65" s="22" t="str" cm="1">
         <f t="array" ref="I65">_xlfn.IFS(LEFT(G65,1)-RIGHT(G65,1) &gt; 0, "W1",LEFT(G65,1)-RIGHT(G65,1) = 0, "D",LEFT(G65,1)-RIGHT(G65,1) &lt; 0, "W2", ISBLANK(G65), "")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J65" s="23" t="e">
+        <v>W1</v>
+      </c>
+      <c r="J65" s="23">
         <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -15052,15 +15072,17 @@
       <c r="F70" s="137" t="s">
         <v>2392</v>
       </c>
-      <c r="G70" s="157"/>
+      <c r="G70" s="157" t="s">
+        <v>2484</v>
+      </c>
       <c r="H70" s="24"/>
-      <c r="I70" s="24" t="e" cm="1">
+      <c r="I70" s="24" t="str" cm="1">
         <f t="array" ref="I70">_xlfn.IFS(LEFT(G70,1)-RIGHT(G70,1) &gt; 0, "W1",LEFT(G70,1)-RIGHT(G70,1) = 0, "D",LEFT(G70,1)-RIGHT(G70,1) &lt; 0, "W2", ISBLANK(G70), "")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J70" s="25" t="e">
+        <v>D</v>
+      </c>
+      <c r="J70" s="25">
         <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.35">
@@ -15082,15 +15104,19 @@
       <c r="F71" s="137" t="s">
         <v>2393</v>
       </c>
-      <c r="G71" s="157"/>
-      <c r="H71" s="24"/>
-      <c r="I71" s="24" t="e" cm="1">
+      <c r="G71" s="157" t="s">
+        <v>2471</v>
+      </c>
+      <c r="H71" s="24" t="s">
+        <v>3845</v>
+      </c>
+      <c r="I71" s="24" t="str" cm="1">
         <f t="array" ref="I71">_xlfn.IFS(LEFT(G71,1)-RIGHT(G71,1) &gt; 0, "W1",LEFT(G71,1)-RIGHT(G71,1) = 0, "D",LEFT(G71,1)-RIGHT(G71,1) &lt; 0, "W2", ISBLANK(G71), "")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J71" s="25" t="e">
+        <v>W2</v>
+      </c>
+      <c r="J71" s="25">
         <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="72" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Upcoming table changes + Lawson's bets
</commit_message>
<xml_diff>
--- a/FIFAScheduleResults.xlsx
+++ b/FIFAScheduleResults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/francis_fayolle_undp_org/Documents/Documents/World-Cup-betting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="460" documentId="13_ncr:1_{AD0E7F59-3B0E-407E-93E9-FE21F83F93C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{577A8126-5436-4E83-AAE9-8E2303267153}"/>
+  <xr:revisionPtr revIDLastSave="461" documentId="13_ncr:1_{AD0E7F59-3B0E-407E-93E9-FE21F83F93C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C678DBE-6D0D-40B0-8B81-AD5097D14663}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12798,7 +12798,7 @@
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="15.81640625" customWidth="1"/>
     <col min="7" max="7" width="30" style="143" customWidth="1"/>
-    <col min="8" max="8" width="38.08984375" style="163" customWidth="1"/>
+    <col min="8" max="8" width="47.81640625" style="163" customWidth="1"/>
     <col min="9" max="9" width="12.26953125" style="163" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>